<commit_message>
test expanding forward look and including pub leads
</commit_message>
<xml_diff>
--- a/Forward Look/Forward Look.xlsx
+++ b/Forward Look/Forward Look.xlsx
@@ -12,12 +12,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
   <si>
     <t xml:space="preserve">MoJ Statistics Forward Look</t>
   </si>
   <si>
-    <t xml:space="preserve">This list contains a week-by-week view of  MoJ Official and National Statistics that have been pre-announced on the gov.uk release calendar as at 14 November 2025</t>
+    <t xml:space="preserve">This list contains a week-by-week view of  MoJ Official and National Statistics that have been pre-announced on the gov.uk release calendar as at 20 November 2025</t>
   </si>
   <si>
     <t xml:space="preserve">Click here to view on the gov.uk Research and Statistics calendar</t>
@@ -41,13 +41,16 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">17 Nov 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Knife and Offensive Weapon Sentencing Statistics:  April to June 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 November 2025</t>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 Nov 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Her Majesty’s Prison and Probation Service Staff Equalities Report: 2024 to 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27 November 2025</t>
   </si>
   <si>
     <t xml:space="preserve">confirmed</t>
@@ -56,36 +59,39 @@
     <t xml:space="preserve">standard</t>
   </si>
   <si>
-    <t xml:space="preserve"> HM Prison and Probation Service workforce quarterly: September 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 Nov 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Her Majesty’s Prison and Probation Service Staff Equalities Report: 2024 to 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 November 2025</t>
+    <t xml:space="preserve">The HMPPS annual Staff Equalities Report considers profiles and processes of the HMPPS workforce from an equalities perspective.</t>
   </si>
   <si>
     <t xml:space="preserve">His Majesty’s Prison and Probation Service offender equalities report: 2024 to 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Equalities-focused tables and commentary encompassing a wide range of issues relating to offenders across prisons and probation.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ethnicity and the Criminal Justice System 2024</t>
   </si>
   <si>
+    <t xml:space="preserve">This report compiles statistics from data sources across the Criminal Justice System, to provide a combined perspective on the typical experiences of different ethnic groups in England and Wales.</t>
+  </si>
+  <si>
     <t xml:space="preserve">01 Dec 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> Civil justice statistics: July to September 2025</t>
+    <t xml:space="preserve">Civil justice statistics: July to September 2025</t>
   </si>
   <si>
     <t xml:space="preserve">4 December 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Volume of civil and judicial review cases dealt with by the courts over time and the overall timeliness of these cases.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Prison Population Projections: 2025 to 2030</t>
   </si>
   <si>
+    <t xml:space="preserve">Five year projections for the population in England and Wales prisons.</t>
+  </si>
+  <si>
     <t xml:space="preserve">08 Dec 2025</t>
   </si>
   <si>
@@ -95,6 +101,9 @@
     <t xml:space="preserve">11 December 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Type and volume of tribunal cases received, disposed of or outstanding. This also includes statistics on the Gender Recognition Certificate applied for and granted by HMCTS Gender Recognition Panel.</t>
+  </si>
+  <si>
     <t xml:space="preserve">15 Dec 2025</t>
   </si>
   <si>
@@ -104,40 +113,64 @@
     <t xml:space="preserve">18 December 2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Volume of cases dealt with by family courts over time, with statistics also broken down for the main types of case involved. Includes data on Children Act cases (both public and private law), Matrimonial matters, Domestic Violence Remedy Orders, Forced Marriage Protection Orders, Female Genital Mutilation Protection Orders, adoptions, The Mental Capacity Act and probate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criminal court statistics quarterly: July to September 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type and volume of cases received and processed through the criminal court system of England and Wales, including statistics on case timeliness. Also includes statistics on the use of language interpreter and translation services in courts and tribunals, England and Wales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legal aid statistics quarterly: July to September 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cancelled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activity in the legal aid system for England and Wales, including criminal and civil legal aid, family mediation, providers of legal aid, client characteristics and Central Funds payments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22 Dec 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">05 Jan 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 Jan 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19 Jan 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26 Jan 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Safety in custody: quarterly update to September 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 January 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quarterly update on deaths, self-harm and assaults in prison custody in England and Wales. Additional annual deaths tables (to 2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02 Feb 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09 Feb 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortgage and landlord possession statistics: October to December 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 February 2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">provisional</t>
   </si>
   <si>
-    <t xml:space="preserve">Criminal court statistics quarterly: July to September 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legal aid statistics quarterly: July to September 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 Dec 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">05 Jan 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12 Jan 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19 Jan 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26 Jan 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Safety in custody: quarterly update to September 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 January 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">02 Feb 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09 Feb 2026</t>
+    <t xml:space="preserve">Quarterly National Statistics on possession claim actions in county courts by mortgage lenders and social and private landlords.</t>
   </si>
   <si>
     <t xml:space="preserve">16 Feb 2026</t>
@@ -230,12 +263,21 @@
     <t xml:space="preserve">30 July 2026</t>
   </si>
   <si>
+    <t xml:space="preserve">Annual release on employment status of offenders post release from custody and on community sentences. Covers employment rates, and those who are unable to work.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Offender accommodation outcomes, update to March 2026</t>
   </si>
   <si>
+    <t xml:space="preserve">Annual release on accommodation status of offenders post release from custody and on community sentences. Covers those who are housed, homeless or rough sleeping.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Community Performance Annual, update to March 2026</t>
   </si>
   <si>
+    <t xml:space="preserve">An annual release of performance statistics for the Probation Service, incorporating Probation Service and Commissioned Rehabilitative Services performance.</t>
+  </si>
+  <si>
     <t xml:space="preserve">03 Aug 2026</t>
   </si>
   <si>
@@ -285,6 +327,9 @@
   </si>
   <si>
     <t xml:space="preserve">29 October 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of deaths of offenders supervised in the community by the Probation Service in England and Wales</t>
   </si>
 </sst>
 </file>
@@ -354,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -364,6 +409,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -718,10 +769,11 @@
   <cols>
     <col min="1" max="1" width="18.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="95.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="30.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="20.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="10.71" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="10.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="60.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,845 +810,907 @@
       <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G4" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" t="n">
         <v>48</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>51</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
       <c r="E14" s="5" t="n">
-        <v>51</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="6"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
       <c r="E15" s="5" t="n">
-        <v>51</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="6"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="n">
-        <v>52</v>
+        <v>3</v>
       </c>
       <c r="F16" s="5"/>
+      <c r="G16" s="6"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="5"/>
+      <c r="G17" s="6"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
+        <v>43</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="E18" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" s="5"/>
+        <v>5</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F19" s="5"/>
+      <c r="G19" s="6"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F21" s="5"/>
+      <c r="G21" s="6"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F22" s="5"/>
+      <c r="G22" s="6"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F23" s="5"/>
+      <c r="G23" s="6"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F24" s="5"/>
+      <c r="G24" s="6"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="5"/>
+      <c r="G25" s="6"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
+        <v>58</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="E26" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F26" s="5"/>
+        <v>13</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F27" s="5"/>
+      <c r="G27" s="6"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
       <c r="E28" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="6"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F29" s="5"/>
+      <c r="G29" s="6"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F30" s="5"/>
+      <c r="G30" s="6"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F31" s="5"/>
+      <c r="G31" s="6"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F32" s="5"/>
+      <c r="G32" s="6"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F33" s="5"/>
+      <c r="G33" s="6"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F34" s="5"/>
+      <c r="G34" s="6"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F35" s="5"/>
+      <c r="G35" s="6"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F36" s="5"/>
+      <c r="G36" s="6"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F37" s="5"/>
+      <c r="G37" s="6"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F38" s="5"/>
+      <c r="G38" s="6"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F39" s="5"/>
+      <c r="G39" s="6"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="5"/>
-      <c r="D40" s="5"/>
+        <v>74</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="E40" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="F40" s="5"/>
+        <v>27</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="5" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F41" s="5"/>
+      <c r="G41" s="6"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
       <c r="E42" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="F42" s="5"/>
+      <c r="G42" s="6"/>
     </row>
     <row r="43">
       <c r="A43" s="5" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="5" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F43" s="5"/>
+      <c r="G43" s="6"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B44" s="5"/>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="E44" s="5" t="n">
-        <v>29</v>
-      </c>
-      <c r="F44" s="5"/>
+        <v>31</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" s="6" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B45" s="5"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="5"/>
+        <v>80</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="E45" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="F45" s="5"/>
+        <v>31</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" s="6" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E46" s="5" t="n">
         <v>31</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="G46" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>12</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="B47" s="5"/>
+      <c r="C47" s="5"/>
+      <c r="D47" s="5"/>
       <c r="E47" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="F47" s="5"/>
+      <c r="G47" s="6"/>
     </row>
     <row r="48">
       <c r="A48" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>12</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
       <c r="E48" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F48" s="5"/>
+      <c r="G48" s="6"/>
     </row>
     <row r="49">
       <c r="A49" s="5" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F49" s="5"/>
+      <c r="G49" s="6"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="B50" s="5"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F50" s="5"/>
+      <c r="G50" s="6"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="B51" s="5"/>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F51" s="5"/>
+      <c r="G51" s="6"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="B52" s="5"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F52" s="5"/>
+      <c r="G52" s="6"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="B53" s="5"/>
       <c r="C53" s="5"/>
       <c r="D53" s="5"/>
       <c r="E53" s="5" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F53" s="5"/>
+      <c r="G53" s="6"/>
     </row>
     <row r="54">
       <c r="A54" s="5" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F54" s="5"/>
+      <c r="G54" s="6"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
+        <v>96</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C55" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>51</v>
+      </c>
       <c r="E55" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="F55" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="B56" s="5"/>
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F56" s="5"/>
+      <c r="G56" s="6"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D57" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
       <c r="E57" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="F57" s="5"/>
+      <c r="G57" s="6"/>
     </row>
     <row r="58">
       <c r="A58" s="5" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B58" s="5"/>
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F58" s="5"/>
+      <c r="G58" s="6"/>
     </row>
     <row r="59">
       <c r="A59" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
+        <v>102</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="E59" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="F59" s="5"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5" t="n">
-        <v>43</v>
-      </c>
-      <c r="F60" s="5"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="F61" s="5" t="s">
-        <v>13</v>
+      <c r="F59" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:F61">
+  <conditionalFormatting sqref="A5:G59">
     <cfRule type="expression" dxfId="0" priority="5">
       <formula>=AND(LEN($E5)&gt;0,MOD(RIGHT($E5,2),2)=0)</formula>
     </cfRule>
@@ -1607,7 +1721,7 @@
       <formula>=AND($E5&lt;&gt;$E4)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A61">
+  <conditionalFormatting sqref="A5:A59">
     <cfRule type="expression" dxfId="2" priority="3">
       <formula>=AND(LEN($E5)&gt;0,MOD(RIGHT($E5,2),2)=0,$E5=$E4)</formula>
     </cfRule>

</xml_diff>